<commit_message>
lower dashboard code update
</commit_message>
<xml_diff>
--- a/data/test_case_selector.xlsx
+++ b/data/test_case_selector.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="840">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="839">
   <si>
     <t>task_name</t>
   </si>
@@ -2544,9 +2544,6 @@
   </si>
   <si>
     <t>Bhavani@12</t>
-  </si>
-  <si>
-    <t>bhavani+38@secmark.in</t>
   </si>
   <si>
     <t>Test QA</t>
@@ -6331,10 +6328,10 @@
     </row>
     <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
-        <v>830</v>
+        <v>693</v>
       </c>
       <c r="B2" s="43" t="s">
-        <v>352</v>
+        <v>694</v>
       </c>
       <c r="C2" s="103" t="s">
         <v>695</v>
@@ -6399,7 +6396,7 @@
         <v>481</v>
       </c>
       <c r="D2" s="94" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -6413,7 +6410,7 @@
         <v>482</v>
       </c>
       <c r="D3" s="94" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -12345,7 +12342,7 @@
         <v>760</v>
       </c>
       <c r="C2" s="50" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D2" s="30">
         <v>46150</v>
@@ -12373,7 +12370,7 @@
         <v>698</v>
       </c>
       <c r="O2" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P2" s="12" t="s">
         <v>39</v>
@@ -12408,7 +12405,7 @@
         <v>761</v>
       </c>
       <c r="C3" s="50" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D3" s="30">
         <v>46150</v>
@@ -12440,7 +12437,7 @@
         <v>698</v>
       </c>
       <c r="O3" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P3" s="12" t="s">
         <v>39</v>
@@ -12475,7 +12472,7 @@
         <v>762</v>
       </c>
       <c r="C4" s="50" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D4" s="30">
         <v>46150</v>
@@ -12509,7 +12506,7 @@
         <v>698</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P4" s="12" t="s">
         <v>39</v>
@@ -12544,7 +12541,7 @@
         <v>763</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D5" s="30">
         <v>46150</v>
@@ -12578,7 +12575,7 @@
         <v>698</v>
       </c>
       <c r="O5" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P5" s="12" t="s">
         <v>39</v>
@@ -12613,7 +12610,7 @@
         <v>764</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D6" s="30">
         <v>46150</v>
@@ -12647,7 +12644,7 @@
         <v>698</v>
       </c>
       <c r="O6" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P6" s="12" t="s">
         <v>39</v>
@@ -12682,7 +12679,7 @@
         <v>765</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D7" s="30">
         <v>46150</v>
@@ -12716,7 +12713,7 @@
         <v>698</v>
       </c>
       <c r="O7" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P7" s="12" t="s">
         <v>39</v>
@@ -12751,7 +12748,7 @@
         <v>766</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D8" s="30">
         <v>46150</v>
@@ -12785,7 +12782,7 @@
         <v>698</v>
       </c>
       <c r="O8" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P8" s="12" t="s">
         <v>39</v>
@@ -12820,7 +12817,7 @@
         <v>767</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D9" s="30">
         <v>46150</v>
@@ -12854,7 +12851,7 @@
         <v>698</v>
       </c>
       <c r="O9" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P9" s="12" t="s">
         <v>39</v>
@@ -15981,7 +15978,7 @@
         <v>153</v>
       </c>
       <c r="C2" s="50" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="D2" s="30">
         <v>46150</v>
@@ -16009,7 +16006,7 @@
         <v>698</v>
       </c>
       <c r="O2" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P2" s="50" t="s">
         <v>39</v>
@@ -16047,7 +16044,7 @@
         <v>761</v>
       </c>
       <c r="C3" s="50" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="D3" s="30">
         <v>46150</v>
@@ -16079,7 +16076,7 @@
         <v>698</v>
       </c>
       <c r="O3" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P3" s="50" t="s">
         <v>39</v>
@@ -16117,7 +16114,7 @@
         <v>762</v>
       </c>
       <c r="C4" s="50" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D4" s="30">
         <v>46150</v>
@@ -16151,7 +16148,7 @@
         <v>698</v>
       </c>
       <c r="O4" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P4" s="50" t="s">
         <v>39</v>
@@ -16189,7 +16186,7 @@
         <v>763</v>
       </c>
       <c r="C5" s="50" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D5" s="30">
         <v>46150</v>
@@ -16223,7 +16220,7 @@
         <v>698</v>
       </c>
       <c r="O5" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P5" s="50" t="s">
         <v>39</v>
@@ -16261,7 +16258,7 @@
         <v>764</v>
       </c>
       <c r="C6" s="50" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D6" s="30">
         <v>46150</v>
@@ -16295,7 +16292,7 @@
         <v>698</v>
       </c>
       <c r="O6" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P6" s="50" t="s">
         <v>39</v>
@@ -16333,7 +16330,7 @@
         <v>765</v>
       </c>
       <c r="C7" s="50" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D7" s="30">
         <v>46150</v>
@@ -16367,7 +16364,7 @@
         <v>698</v>
       </c>
       <c r="O7" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P7" s="50" t="s">
         <v>39</v>
@@ -16405,7 +16402,7 @@
         <v>766</v>
       </c>
       <c r="C8" s="50" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D8" s="30">
         <v>46150</v>
@@ -16439,7 +16436,7 @@
         <v>698</v>
       </c>
       <c r="O8" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P8" s="50" t="s">
         <v>39</v>
@@ -16477,7 +16474,7 @@
         <v>767</v>
       </c>
       <c r="C9" s="50" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D9" s="30">
         <v>46150</v>
@@ -16511,7 +16508,7 @@
         <v>698</v>
       </c>
       <c r="O9" s="46" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="P9" s="50" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
new server changes updated
</commit_message>
<xml_diff>
--- a/data/test_case_selector.xlsx
+++ b/data/test_case_selector.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" activeTab="1"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" firstSheet="7" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="credentials" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2838" uniqueCount="934">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2838" uniqueCount="933">
   <si>
     <t>task_name</t>
   </si>
@@ -2638,9 +2638,6 @@
     <t>rahuld@secmark.in</t>
   </si>
   <si>
-    <t>Test the Task_Only_once 29-06</t>
-  </si>
-  <si>
     <t>bulk_task_creation</t>
   </si>
   <si>
@@ -2848,9 +2845,6 @@
     <t>{"normal_task":"Test Normal Task"}</t>
   </si>
   <si>
-    <t>Test the Task_Only_once 15_07</t>
-  </si>
-  <si>
     <t>{"company_name":"Test Company_1213", "license_name":"BSE"}</t>
   </si>
   <si>
@@ -2858,6 +2852,9 @@
   </si>
   <si>
     <t>{"company_name" : "Test Company_4056", "license_name":"BSE"}</t>
+  </si>
+  <si>
+    <t>Test the Task_Only_once 21-07</t>
   </si>
 </sst>
 </file>
@@ -6552,7 +6549,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="66" customFormat="1" x14ac:dyDescent="0.25">
@@ -6696,7 +6693,7 @@
       </c>
       <c r="E9" s="62"/>
       <c r="F9" s="120" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -7136,16 +7133,16 @@
         <v>820</v>
       </c>
       <c r="B34" s="110" t="s">
+        <v>860</v>
+      </c>
+      <c r="C34" t="s">
         <v>861</v>
-      </c>
-      <c r="C34" t="s">
-        <v>862</v>
       </c>
       <c r="D34" s="82" t="s">
         <v>272</v>
       </c>
       <c r="E34" s="62" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F34" s="66" t="s">
         <v>134</v>
@@ -7177,7 +7174,7 @@
         <v>821</v>
       </c>
       <c r="C36" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="D36" s="82" t="s">
         <v>272</v>
@@ -7191,7 +7188,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="47" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B37" s="115" t="s">
         <v>850</v>
@@ -7209,7 +7206,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="47" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B38" s="115" t="s">
         <v>851</v>
@@ -7227,19 +7224,19 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="47" t="s">
+        <v>902</v>
+      </c>
+      <c r="B39" s="115" t="s">
         <v>903</v>
       </c>
-      <c r="B39" s="115" t="s">
+      <c r="C39" s="140" t="s">
         <v>904</v>
-      </c>
-      <c r="C39" s="140" t="s">
-        <v>905</v>
       </c>
       <c r="D39" s="116" t="s">
         <v>272</v>
       </c>
       <c r="E39" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="F39" s="66" t="s">
         <v>134</v>
@@ -7247,22 +7244,22 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="47" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B40" s="47" t="s">
         <v>619</v>
       </c>
       <c r="C40" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="D40" s="67" t="s">
         <v>272</v>
       </c>
       <c r="E40" s="66" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F40" s="120" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -7323,7 +7320,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -7730,7 +7727,7 @@
         <v>528</v>
       </c>
       <c r="C24" s="139" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="D24" s="82" t="s">
         <v>272</v>
@@ -7781,16 +7778,16 @@
         <v>521</v>
       </c>
       <c r="B27" s="110" t="s">
+        <v>860</v>
+      </c>
+      <c r="C27" t="s">
         <v>861</v>
-      </c>
-      <c r="C27" t="s">
-        <v>862</v>
       </c>
       <c r="D27" s="82" t="s">
         <v>272</v>
       </c>
       <c r="E27" s="62" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="F27" s="66" t="s">
         <v>134</v>
@@ -7888,7 +7885,7 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="86" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B33" s="82" t="s">
         <v>460</v>
@@ -7906,19 +7903,19 @@
     </row>
     <row r="34" spans="1:6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="86" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="B34" s="115" t="s">
         <v>831</v>
       </c>
       <c r="C34" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="D34" s="116" t="s">
         <v>272</v>
       </c>
       <c r="E34" s="62" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="F34" s="66" t="s">
         <v>134</v>
@@ -7926,19 +7923,19 @@
     </row>
     <row r="35" spans="1:6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="86" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="B35" s="47" t="s">
         <v>632</v>
       </c>
       <c r="C35" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="D35" s="70" t="s">
         <v>272</v>
       </c>
       <c r="E35" s="66" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="F35" s="66" t="s">
         <v>133</v>
@@ -8024,7 +8021,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -8462,7 +8459,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -8729,7 +8726,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
@@ -8740,7 +8737,7 @@
         <v>855</v>
       </c>
       <c r="C2" s="87" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="D2" s="67" t="s">
         <v>272</v>
@@ -8757,7 +8754,7 @@
         <v>856</v>
       </c>
       <c r="C3" s="87" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="D3" t="s">
         <v>272</v>
@@ -8922,7 +8919,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -9269,7 +9266,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -9440,7 +9437,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -9485,7 +9482,7 @@
         <v>711</v>
       </c>
       <c r="C4" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="D4" s="47" t="s">
         <v>272</v>
@@ -9502,7 +9499,7 @@
         <v>719</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>272</v>
@@ -9550,7 +9547,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -9671,7 +9668,7 @@
         <v>832</v>
       </c>
       <c r="C8" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="D8" s="118" t="s">
         <v>272</v>
@@ -9719,7 +9716,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -9730,7 +9727,7 @@
         <v>564</v>
       </c>
       <c r="C2" s="62" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="D2" s="47" t="s">
         <v>272</v>
@@ -9750,7 +9747,7 @@
         <v>593</v>
       </c>
       <c r="C3" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="D3" s="47" t="s">
         <v>272</v>
@@ -9822,7 +9819,7 @@
         <v>666</v>
       </c>
       <c r="C7" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>272</v>
@@ -9842,7 +9839,7 @@
         <v>665</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>272</v>
@@ -9942,7 +9939,7 @@
         <v>757</v>
       </c>
       <c r="C13" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="D13" s="47" t="s">
         <v>272</v>
@@ -9960,7 +9957,7 @@
         <v>686</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="D14" s="47" t="s">
         <v>272</v>
@@ -9978,7 +9975,7 @@
         <v>627</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="D15" s="47" t="s">
         <v>272</v>
@@ -9998,7 +9995,7 @@
         <v>628</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="D16" s="47" t="s">
         <v>272</v>
@@ -10018,7 +10015,7 @@
         <v>626</v>
       </c>
       <c r="C17" s="107" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="D17" s="104" t="s">
         <v>272</v>
@@ -10154,7 +10151,7 @@
         <v>128</v>
       </c>
       <c r="B8" s="44" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C8" s="44" t="s">
         <v>133</v>
@@ -10308,7 +10305,7 @@
         <v>599</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C19" s="95" t="s">
         <v>133</v>
@@ -10366,7 +10363,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -10526,7 +10523,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -10632,7 +10629,7 @@
         <v>629</v>
       </c>
       <c r="B7" s="47" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="C7" t="s">
         <v>701</v>
@@ -10641,7 +10638,7 @@
         <v>272</v>
       </c>
       <c r="E7" s="62" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="F7" s="120" t="s">
         <v>133</v>
@@ -10661,7 +10658,7 @@
         <v>272</v>
       </c>
       <c r="E8" s="62" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="F8" s="120" t="s">
         <v>134</v>
@@ -10776,7 +10773,7 @@
         <v>272</v>
       </c>
       <c r="E14" s="62" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="F14" s="120" t="s">
         <v>134</v>
@@ -10804,10 +10801,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="110" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B16" s="141" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C16" s="88" t="s">
         <v>547</v>
@@ -10821,13 +10818,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="110" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="B17" s="141" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C17" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="D17" s="141" t="s">
         <v>272</v>
@@ -10838,13 +10835,13 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="110" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="B18" s="141" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C18" s="88" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="D18" s="141" t="s">
         <v>272</v>
@@ -13399,7 +13396,7 @@
         <v>602</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" x14ac:dyDescent="0.25">
@@ -13500,10 +13497,10 @@
     </row>
     <row r="17" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C17" s="66"/>
       <c r="D17" s="66"/>
@@ -29924,7 +29921,7 @@
         <v>633</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="23" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29948,7 +29945,7 @@
         <v>635</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="26" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29964,7 +29961,7 @@
         <v>656</v>
       </c>
       <c r="B27" s="44" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="28" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29972,7 +29969,7 @@
         <v>644</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="29" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29980,7 +29977,7 @@
         <v>643</v>
       </c>
       <c r="B29" s="38" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
     </row>
     <row r="30" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29988,7 +29985,7 @@
         <v>645</v>
       </c>
       <c r="B30" s="44" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
     </row>
     <row r="31" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30053,12 +30050,12 @@
         <v>136</v>
       </c>
       <c r="F1" s="72" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B2" s="121" t="s">
         <v>137</v>
@@ -30078,7 +30075,7 @@
     </row>
     <row r="3" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B3" s="118" t="s">
         <v>312</v>
@@ -30098,7 +30095,7 @@
     </row>
     <row r="4" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B4" s="51" t="s">
         <v>142</v>
@@ -30118,7 +30115,7 @@
     </row>
     <row r="5" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B5" s="118" t="s">
         <v>138</v>
@@ -30138,7 +30135,7 @@
     </row>
     <row r="6" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B6" s="51" t="s">
         <v>309</v>
@@ -30158,7 +30155,7 @@
     </row>
     <row r="7" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B7" s="48" t="s">
         <v>140</v>
@@ -30176,7 +30173,7 @@
     </row>
     <row r="8" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B8" s="51" t="s">
         <v>141</v>
@@ -30194,7 +30191,7 @@
     </row>
     <row r="9" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B9" s="48" t="s">
         <v>139</v>
@@ -30210,7 +30207,7 @@
     </row>
     <row r="10" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B10" s="51" t="s">
         <v>314</v>
@@ -30230,7 +30227,7 @@
     </row>
     <row r="11" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B11" s="48" t="s">
         <v>313</v>
@@ -30387,7 +30384,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="122" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -30648,7 +30645,7 @@
         <v>136</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:6" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -31106,7 +31103,7 @@
         <v>136</v>
       </c>
       <c r="X1" s="124" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -31117,13 +31114,13 @@
         <v>729</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="D2" s="30">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="E2" s="30">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>104</v>
@@ -31183,7 +31180,7 @@
         <v>730</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D3" s="30">
         <v>46218</v>
@@ -31253,7 +31250,7 @@
         <v>731</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D4" s="30">
         <v>46218</v>
@@ -31325,7 +31322,7 @@
         <v>732</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D5" s="30">
         <v>46218</v>
@@ -31397,7 +31394,7 @@
         <v>733</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D6" s="30">
         <v>46218</v>
@@ -31469,7 +31466,7 @@
         <v>734</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D7" s="30">
         <v>46218</v>
@@ -31541,7 +31538,7 @@
         <v>735</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D8" s="30">
         <v>46218</v>
@@ -31613,7 +31610,7 @@
         <v>736</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="D9" s="30">
         <v>46218</v>
@@ -34876,7 +34873,7 @@
         <v>136</v>
       </c>
       <c r="Y1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -34887,13 +34884,13 @@
         <v>150</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>860</v>
+        <v>932</v>
       </c>
       <c r="D2" s="30">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="E2" s="30">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>104</v>
@@ -34956,7 +34953,7 @@
         <v>730</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D3" s="30">
         <v>46211</v>
@@ -35029,7 +35026,7 @@
         <v>731</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D4" s="30">
         <v>46211</v>
@@ -35104,7 +35101,7 @@
         <v>732</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D5" s="30">
         <v>46211</v>
@@ -35179,7 +35176,7 @@
         <v>733</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D6" s="30">
         <v>46211</v>
@@ -35254,7 +35251,7 @@
         <v>734</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D7" s="30">
         <v>46211</v>
@@ -35329,7 +35326,7 @@
         <v>735</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D8" s="30">
         <v>46211</v>
@@ -35404,7 +35401,7 @@
         <v>736</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="D9" s="30">
         <v>46211</v>
@@ -39062,7 +39059,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="2" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Working on Audit Company
</commit_message>
<xml_diff>
--- a/data/test_case_selector.xlsx
+++ b/data/test_case_selector.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10305" firstSheet="19" activeTab="21"/>
   </bookViews>
   <sheets>
     <sheet name="credentials" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,8 @@
     <sheet name="project_test_cases" sheetId="19" r:id="rId19"/>
     <sheet name="normal_task_sections_test_cases" sheetId="15" r:id="rId20"/>
     <sheet name="settings_test_cases" sheetId="17" r:id="rId21"/>
-    <sheet name="helper" sheetId="8" r:id="rId22"/>
+    <sheet name="audit_test_cases" sheetId="26" r:id="rId22"/>
+    <sheet name="helper" sheetId="8" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">dashboard_test_cases!$A$1:$D$26</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="939">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2886" uniqueCount="959">
   <si>
     <t>task_name</t>
   </si>
@@ -2209,9 +2210,6 @@
     <t>Verify that column filters in Compliance Events work correctly using the first available values.</t>
   </si>
   <si>
-    <t>Verify that the Issuer link and Dashboard are clickable and navigate to the correct pages</t>
-  </si>
-  <si>
     <t>Verify that a task can be created under "Create Your Own Task" in Updates and is displayed on the Dashboard.</t>
   </si>
   <si>
@@ -2873,6 +2871,69 @@
   </si>
   <si>
     <t>preprod</t>
+  </si>
+  <si>
+    <t>TC_Settings_18</t>
+  </si>
+  <si>
+    <t>bulk_invitations</t>
+  </si>
+  <si>
+    <t>Verify bulk Invitations using Excel file upload</t>
+  </si>
+  <si>
+    <t>TC_Settings_19</t>
+  </si>
+  <si>
+    <t>bulk_invitation_download_template</t>
+  </si>
+  <si>
+    <t>Verify that the Issuer link and Download are clickable and navigate to the correct pages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify bulk Invitation download is clickable </t>
+  </si>
+  <si>
+    <t>audit</t>
+  </si>
+  <si>
+    <t>audit_company</t>
+  </si>
+  <si>
+    <t>verify audit company details</t>
+  </si>
+  <si>
+    <t>TC_Audit_1</t>
+  </si>
+  <si>
+    <t>bhavani+69@secmark.in</t>
+  </si>
+  <si>
+    <t>{"email_id" : "testuser234@gmail.com"}</t>
+  </si>
+  <si>
+    <t>TC_Audit_2</t>
+  </si>
+  <si>
+    <t>audit_branch</t>
+  </si>
+  <si>
+    <t>verify audit branch details</t>
+  </si>
+  <si>
+    <t>TC_Audit_3</t>
+  </si>
+  <si>
+    <t>verify Export data details</t>
+  </si>
+  <si>
+    <t>TC_Audit_4</t>
+  </si>
+  <si>
+    <t>search_company_name</t>
+  </si>
+  <si>
+    <t>verify search company name  data details</t>
   </si>
 </sst>
 </file>
@@ -2885,7 +2946,7 @@
     <numFmt numFmtId="166" formatCode="dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="167" formatCode="d\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3038,6 +3099,18 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -3429,7 +3502,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3781,6 +3854,12 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -6054,8 +6133,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="A1:D20" totalsRowShown="0" headerRowDxfId="119" dataDxfId="118">
-  <autoFilter ref="A1:D20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Table7" displayName="Table7" ref="A1:D21" totalsRowShown="0" headerRowDxfId="119" dataDxfId="118">
+  <autoFilter ref="A1:D21"/>
   <tableColumns count="4">
     <tableColumn id="3" name="module_to_test" dataDxfId="117"/>
     <tableColumn id="4" name="execution" dataDxfId="116"/>
@@ -6507,24 +6586,24 @@
         <v>586</v>
       </c>
       <c r="E1" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
-        <v>859</v>
+        <v>949</v>
       </c>
       <c r="B2" s="41" t="s">
-        <v>670</v>
+        <v>339</v>
       </c>
       <c r="C2" s="91" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D2" s="93" t="s">
         <v>587</v>
       </c>
       <c r="E2" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -6577,7 +6656,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="66" customFormat="1" x14ac:dyDescent="0.25">
@@ -7158,19 +7237,19 @@
     </row>
     <row r="34" spans="1:6" s="66" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="47" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B34" s="110" t="s">
+        <v>859</v>
+      </c>
+      <c r="C34" t="s">
         <v>860</v>
-      </c>
-      <c r="C34" t="s">
-        <v>861</v>
       </c>
       <c r="D34" s="82" t="s">
         <v>272</v>
       </c>
       <c r="E34" s="62" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F34" s="66" t="s">
         <v>134</v>
@@ -7178,7 +7257,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="47" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="B35" s="110" t="s">
         <v>713</v>
@@ -7196,19 +7275,19 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="47" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="B36" s="115" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="C36" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="D36" s="82" t="s">
         <v>272</v>
       </c>
       <c r="E36" s="62" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="F36" s="66" t="s">
         <v>134</v>
@@ -7216,10 +7295,10 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="47" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="B37" s="115" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="C37" s="88" t="s">
         <v>540</v>
@@ -7234,10 +7313,10 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="47" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="B38" s="115" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="C38" s="88" t="s">
         <v>491</v>
@@ -7252,19 +7331,19 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="47" t="s">
+        <v>901</v>
+      </c>
+      <c r="B39" s="115" t="s">
         <v>902</v>
       </c>
-      <c r="B39" s="115" t="s">
+      <c r="C39" s="140" t="s">
         <v>903</v>
-      </c>
-      <c r="C39" s="140" t="s">
-        <v>904</v>
       </c>
       <c r="D39" s="116" t="s">
         <v>272</v>
       </c>
       <c r="E39" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="F39" s="66" t="s">
         <v>134</v>
@@ -7272,19 +7351,19 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="47" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="B40" s="47" t="s">
         <v>619</v>
       </c>
       <c r="C40" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="D40" s="67" t="s">
         <v>272</v>
       </c>
       <c r="E40" s="66" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="F40" s="120" t="s">
         <v>134</v>
@@ -7348,7 +7427,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -7374,7 +7453,7 @@
         <v>497</v>
       </c>
       <c r="B3" s="82" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C3" s="83" t="s">
         <v>469</v>
@@ -7410,7 +7489,7 @@
         <v>499</v>
       </c>
       <c r="B5" s="82" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="C5" s="83" t="s">
         <v>475</v>
@@ -7755,7 +7834,7 @@
         <v>528</v>
       </c>
       <c r="C24" s="139" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="D24" s="82" t="s">
         <v>272</v>
@@ -7806,16 +7885,16 @@
         <v>521</v>
       </c>
       <c r="B27" s="110" t="s">
+        <v>859</v>
+      </c>
+      <c r="C27" t="s">
         <v>860</v>
-      </c>
-      <c r="C27" t="s">
-        <v>861</v>
       </c>
       <c r="D27" s="82" t="s">
         <v>272</v>
       </c>
       <c r="E27" s="62" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="F27" s="66" t="s">
         <v>134</v>
@@ -7913,7 +7992,7 @@
     </row>
     <row r="33" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="86" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="B33" s="82" t="s">
         <v>460</v>
@@ -7931,19 +8010,19 @@
     </row>
     <row r="34" spans="1:6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="86" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="B34" s="115" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="C34" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="D34" s="116" t="s">
         <v>272</v>
       </c>
       <c r="E34" s="62" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="F34" s="66" t="s">
         <v>134</v>
@@ -7951,19 +8030,19 @@
     </row>
     <row r="35" spans="1:6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="86" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="B35" s="47" t="s">
         <v>632</v>
       </c>
       <c r="C35" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="D35" s="70" t="s">
         <v>272</v>
       </c>
       <c r="E35" s="66" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="F35" s="66" t="s">
         <v>134</v>
@@ -7971,13 +8050,13 @@
     </row>
     <row r="36" spans="1:6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="86" t="s">
+        <v>933</v>
+      </c>
+      <c r="B36" s="47" t="s">
         <v>934</v>
       </c>
-      <c r="B36" s="47" t="s">
+      <c r="C36" t="s">
         <v>935</v>
-      </c>
-      <c r="C36" t="s">
-        <v>936</v>
       </c>
       <c r="D36" s="70" t="s">
         <v>272</v>
@@ -8064,7 +8143,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -8502,7 +8581,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -8527,7 +8606,7 @@
         <v>297</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="C3" t="s">
         <v>424</v>
@@ -8561,7 +8640,7 @@
         <v>302</v>
       </c>
       <c r="B5" s="47" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="C5" s="48" t="s">
         <v>285</v>
@@ -8578,7 +8657,7 @@
         <v>304</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C6" s="46" t="s">
         <v>307</v>
@@ -8595,7 +8674,7 @@
         <v>305</v>
       </c>
       <c r="B7" s="47" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="C7" s="62" t="s">
         <v>284</v>
@@ -8612,7 +8691,7 @@
         <v>306</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="C8" s="62" t="s">
         <v>594</v>
@@ -8769,18 +8848,18 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
+        <v>853</v>
+      </c>
+      <c r="B2" s="47" t="s">
         <v>854</v>
       </c>
-      <c r="B2" s="47" t="s">
-        <v>855</v>
-      </c>
       <c r="C2" s="87" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="D2" s="67" t="s">
         <v>272</v>
@@ -8791,19 +8870,19 @@
     </row>
     <row r="3" spans="1:6" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="55" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B3" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="C3" s="87" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="D3" t="s">
         <v>272</v>
       </c>
       <c r="E3" s="105" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="F3" s="66" t="s">
         <v>133</v>
@@ -8962,7 +9041,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
@@ -9309,7 +9388,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -9317,10 +9396,10 @@
         <v>552</v>
       </c>
       <c r="B2" s="47" t="s">
+        <v>764</v>
+      </c>
+      <c r="C2" s="47" t="s">
         <v>765</v>
-      </c>
-      <c r="C2" s="47" t="s">
-        <v>766</v>
       </c>
       <c r="D2" s="47" t="s">
         <v>272</v>
@@ -9334,10 +9413,10 @@
         <v>553</v>
       </c>
       <c r="B3" s="113" t="s">
+        <v>766</v>
+      </c>
+      <c r="C3" s="113" t="s">
         <v>767</v>
-      </c>
-      <c r="C3" s="113" t="s">
-        <v>768</v>
       </c>
       <c r="D3" s="47" t="s">
         <v>272</v>
@@ -9351,10 +9430,10 @@
         <v>554</v>
       </c>
       <c r="B4" s="47" t="s">
+        <v>768</v>
+      </c>
+      <c r="C4" s="113" t="s">
         <v>769</v>
-      </c>
-      <c r="C4" s="113" t="s">
-        <v>770</v>
       </c>
       <c r="D4" s="47" t="s">
         <v>272</v>
@@ -9368,10 +9447,10 @@
         <v>555</v>
       </c>
       <c r="B5" s="47" t="s">
+        <v>770</v>
+      </c>
+      <c r="C5" s="113" t="s">
         <v>771</v>
-      </c>
-      <c r="C5" s="113" t="s">
-        <v>772</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>272</v>
@@ -9385,10 +9464,10 @@
         <v>556</v>
       </c>
       <c r="B6" s="47" t="s">
+        <v>772</v>
+      </c>
+      <c r="C6" s="113" t="s">
         <v>773</v>
-      </c>
-      <c r="C6" s="113" t="s">
-        <v>774</v>
       </c>
       <c r="D6" s="47" t="s">
         <v>272</v>
@@ -9402,10 +9481,10 @@
         <v>557</v>
       </c>
       <c r="B7" s="47" t="s">
+        <v>774</v>
+      </c>
+      <c r="C7" s="113" t="s">
         <v>775</v>
-      </c>
-      <c r="C7" s="113" t="s">
-        <v>776</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>272</v>
@@ -9419,10 +9498,10 @@
         <v>558</v>
       </c>
       <c r="B8" s="47" t="s">
+        <v>776</v>
+      </c>
+      <c r="C8" s="113" t="s">
         <v>777</v>
-      </c>
-      <c r="C8" s="113" t="s">
-        <v>778</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>272</v>
@@ -9480,7 +9559,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -9491,7 +9570,7 @@
         <v>695</v>
       </c>
       <c r="C2" s="88" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="D2" s="47" t="s">
         <v>272</v>
@@ -9525,7 +9604,7 @@
         <v>711</v>
       </c>
       <c r="C4" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="D4" s="47" t="s">
         <v>272</v>
@@ -9536,13 +9615,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B5" s="47" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>272</v>
@@ -9590,7 +9669,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -9607,7 +9686,7 @@
         <v>272</v>
       </c>
       <c r="E2" s="47" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="F2" s="66" t="s">
         <v>134</v>
@@ -9639,7 +9718,7 @@
         <v>682</v>
       </c>
       <c r="C4" t="s">
-        <v>717</v>
+        <v>943</v>
       </c>
       <c r="D4" s="118" t="s">
         <v>272</v>
@@ -9657,13 +9736,13 @@
         <v>577</v>
       </c>
       <c r="C5" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="D5" s="118" t="s">
         <v>272</v>
       </c>
       <c r="E5" s="62" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="F5" s="66" t="s">
         <v>134</v>
@@ -9708,10 +9787,10 @@
         <v>683</v>
       </c>
       <c r="B8" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="C8" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="D8" s="118" t="s">
         <v>272</v>
@@ -9759,7 +9838,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -9770,13 +9849,13 @@
         <v>564</v>
       </c>
       <c r="C2" s="62" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="D2" s="47" t="s">
         <v>272</v>
       </c>
       <c r="E2" s="105" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="F2" s="66" t="s">
         <v>134</v>
@@ -9790,7 +9869,7 @@
         <v>593</v>
       </c>
       <c r="C3" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="D3" s="47" t="s">
         <v>272</v>
@@ -9805,7 +9884,7 @@
         <v>615</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="C4" s="88" t="s">
         <v>540</v>
@@ -9823,10 +9902,10 @@
         <v>624</v>
       </c>
       <c r="B5" s="47" t="s">
+        <v>721</v>
+      </c>
+      <c r="C5" s="88" t="s">
         <v>722</v>
-      </c>
-      <c r="C5" s="88" t="s">
-        <v>723</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>272</v>
@@ -9841,7 +9920,7 @@
         <v>625</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="C6" s="88" t="s">
         <v>547</v>
@@ -9862,13 +9941,13 @@
         <v>666</v>
       </c>
       <c r="C7" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>272</v>
       </c>
       <c r="E7" s="108" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="F7" s="66" t="s">
         <v>134</v>
@@ -9882,13 +9961,13 @@
         <v>665</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>272</v>
       </c>
       <c r="E8" s="105" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F8" s="120" t="s">
         <v>134</v>
@@ -9908,7 +9987,7 @@
         <v>272</v>
       </c>
       <c r="E9" s="108" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="F9" s="120" t="s">
         <v>134</v>
@@ -9928,7 +10007,7 @@
         <v>272</v>
       </c>
       <c r="E10" s="105" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="F10" s="120" t="s">
         <v>134</v>
@@ -9939,7 +10018,7 @@
         <v>691</v>
       </c>
       <c r="B11" s="47" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="C11" s="62" t="s">
         <v>617</v>
@@ -9948,7 +10027,7 @@
         <v>272</v>
       </c>
       <c r="E11" s="108" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="F11" s="120" t="s">
         <v>134</v>
@@ -9968,7 +10047,7 @@
         <v>272</v>
       </c>
       <c r="E12" s="105" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="F12" s="120" t="s">
         <v>134</v>
@@ -9976,13 +10055,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="55" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B13" s="47" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C13" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="D13" s="47" t="s">
         <v>272</v>
@@ -9994,13 +10073,13 @@
     </row>
     <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="55" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B14" s="47" t="s">
         <v>686</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="D14" s="47" t="s">
         <v>272</v>
@@ -10012,19 +10091,19 @@
     </row>
     <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="55" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B15" s="47" t="s">
         <v>627</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="D15" s="47" t="s">
         <v>272</v>
       </c>
       <c r="E15" s="105" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="F15" s="120" t="s">
         <v>133</v>
@@ -10032,19 +10111,19 @@
     </row>
     <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="B16" s="47" t="s">
         <v>628</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="D16" s="47" t="s">
         <v>272</v>
       </c>
       <c r="E16" s="108" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="F16" s="120" t="s">
         <v>133</v>
@@ -10052,13 +10131,13 @@
     </row>
     <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="B17" s="104" t="s">
         <v>626</v>
       </c>
       <c r="C17" s="107" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="D17" s="104" t="s">
         <v>272</v>
@@ -10081,7 +10160,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="17.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.5703125" style="39" bestFit="1" customWidth="1"/>
@@ -10177,7 +10256,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="39" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B7" s="44" t="s">
         <v>134</v>
@@ -10208,7 +10287,7 @@
         <v>535</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C9" s="44" t="s">
         <v>133</v>
@@ -10247,7 +10326,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="39" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="B12" s="44" t="s">
         <v>134</v>
@@ -10359,7 +10438,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="39" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B20" s="44" t="s">
         <v>134</v>
@@ -10368,6 +10447,20 @@
         <v>133</v>
       </c>
       <c r="D20" s="114" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="143" t="s">
+        <v>945</v>
+      </c>
+      <c r="B21" s="144" t="s">
+        <v>133</v>
+      </c>
+      <c r="C21" s="144" t="s">
+        <v>133</v>
+      </c>
+      <c r="D21" s="144" t="s">
         <v>134</v>
       </c>
     </row>
@@ -10406,7 +10499,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -10538,7 +10631,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -10566,7 +10659,7 @@
         <v>606</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -10601,7 +10694,7 @@
         <v>272</v>
       </c>
       <c r="E3" s="62" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="F3" s="66" t="s">
         <v>134</v>
@@ -10621,7 +10714,7 @@
         <v>272</v>
       </c>
       <c r="E4" s="62" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="F4" s="66" t="s">
         <v>134</v>
@@ -10641,7 +10734,7 @@
         <v>272</v>
       </c>
       <c r="E5" s="62" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="F5" s="66" t="s">
         <v>134</v>
@@ -10661,7 +10754,7 @@
         <v>272</v>
       </c>
       <c r="E6" s="62" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="F6" s="120" t="s">
         <v>134</v>
@@ -10672,7 +10765,7 @@
         <v>629</v>
       </c>
       <c r="B7" s="47" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C7" t="s">
         <v>701</v>
@@ -10681,7 +10774,7 @@
         <v>272</v>
       </c>
       <c r="E7" s="62" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="F7" s="120" t="s">
         <v>134</v>
@@ -10701,7 +10794,7 @@
         <v>272</v>
       </c>
       <c r="E8" s="62" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="F8" s="120" t="s">
         <v>134</v>
@@ -10759,7 +10852,7 @@
         <v>272</v>
       </c>
       <c r="E11" s="111" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="F11" s="120" t="s">
         <v>134</v>
@@ -10767,13 +10860,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="110" t="s">
+        <v>762</v>
+      </c>
+      <c r="B12" s="110" t="s">
+        <v>761</v>
+      </c>
+      <c r="C12" s="88" t="s">
         <v>763</v>
-      </c>
-      <c r="B12" s="110" t="s">
-        <v>762</v>
-      </c>
-      <c r="C12" s="88" t="s">
-        <v>764</v>
       </c>
       <c r="D12" s="110" t="s">
         <v>272</v>
@@ -10784,19 +10877,19 @@
     </row>
     <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="110" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B13" s="110" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C13" s="88" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D13" s="110" t="s">
         <v>272</v>
       </c>
       <c r="E13" s="62" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="F13" s="120" t="s">
         <v>134</v>
@@ -10804,19 +10897,19 @@
     </row>
     <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="110" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="B14" s="53" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="C14" s="88" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D14" s="53" t="s">
         <v>272</v>
       </c>
       <c r="E14" s="62" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="F14" s="120" t="s">
         <v>134</v>
@@ -10824,30 +10917,30 @@
     </row>
     <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="110" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B15" s="109" t="s">
+        <v>778</v>
+      </c>
+      <c r="C15" s="109" t="s">
         <v>779</v>
-      </c>
-      <c r="C15" s="109" t="s">
-        <v>780</v>
       </c>
       <c r="D15" s="109" t="s">
         <v>272</v>
       </c>
       <c r="E15" s="128" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="F15" s="120" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="110" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="B16" s="141" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C16" s="88" t="s">
         <v>547</v>
@@ -10861,13 +10954,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="110" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="B17" s="141" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C17" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="D17" s="141" t="s">
         <v>272</v>
@@ -10878,19 +10971,53 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="110" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="B18" s="141" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C18" s="88" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="D18" s="141" t="s">
         <v>272</v>
       </c>
       <c r="F18" s="120" t="s">
         <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="110" t="s">
+        <v>938</v>
+      </c>
+      <c r="B19" s="141" t="s">
+        <v>939</v>
+      </c>
+      <c r="C19" t="s">
+        <v>940</v>
+      </c>
+      <c r="D19" s="141" t="s">
+        <v>272</v>
+      </c>
+      <c r="F19" s="120" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="110" t="s">
+        <v>941</v>
+      </c>
+      <c r="B20" s="141" t="s">
+        <v>942</v>
+      </c>
+      <c r="C20" t="s">
+        <v>944</v>
+      </c>
+      <c r="D20" s="141" t="s">
+        <v>272</v>
+      </c>
+      <c r="F20" s="120" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -10903,6 +11030,118 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="93" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="119" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="119" t="s">
+        <v>274</v>
+      </c>
+      <c r="C1" s="119" t="s">
+        <v>271</v>
+      </c>
+      <c r="D1" s="119" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="119" t="s">
+        <v>606</v>
+      </c>
+      <c r="F1" s="119" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="47" t="s">
+        <v>948</v>
+      </c>
+      <c r="B2" s="82" t="s">
+        <v>946</v>
+      </c>
+      <c r="C2" t="s">
+        <v>947</v>
+      </c>
+      <c r="D2" s="82" t="s">
+        <v>272</v>
+      </c>
+      <c r="E2" s="47" t="s">
+        <v>950</v>
+      </c>
+      <c r="F2" s="66" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="47" t="s">
+        <v>951</v>
+      </c>
+      <c r="B3" s="82" t="s">
+        <v>952</v>
+      </c>
+      <c r="C3" t="s">
+        <v>953</v>
+      </c>
+      <c r="D3" s="82" t="s">
+        <v>272</v>
+      </c>
+      <c r="E3" s="47"/>
+      <c r="F3" s="66" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="47" t="s">
+        <v>954</v>
+      </c>
+      <c r="B4" s="82" t="s">
+        <v>293</v>
+      </c>
+      <c r="C4" t="s">
+        <v>955</v>
+      </c>
+      <c r="D4" s="82" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" s="47"/>
+      <c r="F4" s="66" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="47" t="s">
+        <v>956</v>
+      </c>
+      <c r="B5" s="82" t="s">
+        <v>957</v>
+      </c>
+      <c r="C5" t="s">
+        <v>958</v>
+      </c>
+      <c r="D5" s="82" t="s">
+        <v>272</v>
+      </c>
+      <c r="E5" s="47"/>
+      <c r="F5" s="66" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
@@ -13423,7 +13662,7 @@
         <v>93</v>
       </c>
       <c r="B2" s="96" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="17.25" x14ac:dyDescent="0.25">
@@ -13439,7 +13678,7 @@
         <v>602</v>
       </c>
       <c r="B4" s="44" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="17.25" x14ac:dyDescent="0.25">
@@ -13540,10 +13779,10 @@
     </row>
     <row r="17" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="B17" s="44" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C17" s="66"/>
       <c r="D17" s="66"/>
@@ -29964,7 +30203,7 @@
         <v>633</v>
       </c>
       <c r="B22" s="44" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
     </row>
     <row r="23" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29980,7 +30219,7 @@
         <v>639</v>
       </c>
       <c r="B24" s="44" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
     </row>
     <row r="25" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -29988,7 +30227,7 @@
         <v>635</v>
       </c>
       <c r="B25" s="44" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
     </row>
     <row r="26" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30004,7 +30243,7 @@
         <v>656</v>
       </c>
       <c r="B27" s="44" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
     </row>
     <row r="28" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30012,7 +30251,7 @@
         <v>644</v>
       </c>
       <c r="B28" s="44" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
     </row>
     <row r="29" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30020,7 +30259,7 @@
         <v>643</v>
       </c>
       <c r="B29" s="38" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
     </row>
     <row r="30" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30028,7 +30267,7 @@
         <v>645</v>
       </c>
       <c r="B30" s="44" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
     </row>
     <row r="31" spans="1:16384" ht="17.25" x14ac:dyDescent="0.25">
@@ -30093,12 +30332,12 @@
         <v>136</v>
       </c>
       <c r="F1" s="72" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B2" s="121" t="s">
         <v>137</v>
@@ -30118,7 +30357,7 @@
     </row>
     <row r="3" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B3" s="118" t="s">
         <v>312</v>
@@ -30138,7 +30377,7 @@
     </row>
     <row r="4" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="B4" s="51" t="s">
         <v>142</v>
@@ -30158,7 +30397,7 @@
     </row>
     <row r="5" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B5" s="118" t="s">
         <v>138</v>
@@ -30178,7 +30417,7 @@
     </row>
     <row r="6" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="B6" s="51" t="s">
         <v>309</v>
@@ -30198,7 +30437,7 @@
     </row>
     <row r="7" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="B7" s="48" t="s">
         <v>140</v>
@@ -30216,7 +30455,7 @@
     </row>
     <row r="8" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="B8" s="51" t="s">
         <v>141</v>
@@ -30234,7 +30473,7 @@
     </row>
     <row r="9" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="B9" s="48" t="s">
         <v>139</v>
@@ -30250,7 +30489,7 @@
     </row>
     <row r="10" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="B10" s="51" t="s">
         <v>314</v>
@@ -30270,7 +30509,7 @@
     </row>
     <row r="11" spans="1:6" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="B11" s="48" t="s">
         <v>313</v>
@@ -30427,7 +30666,7 @@
         <v>136</v>
       </c>
       <c r="E1" s="122" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -30688,7 +30927,7 @@
         <v>136</v>
       </c>
       <c r="F1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:6" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -30699,7 +30938,7 @@
         <v>319</v>
       </c>
       <c r="C2" s="117" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="D2" s="47">
         <v>1</v>
@@ -30719,7 +30958,7 @@
         <v>310</v>
       </c>
       <c r="C3" s="117" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="D3" s="47">
         <v>1</v>
@@ -30739,7 +30978,7 @@
         <v>311</v>
       </c>
       <c r="C4" s="117" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="D4" s="47">
         <v>0</v>
@@ -30759,7 +30998,7 @@
         <v>148</v>
       </c>
       <c r="C5" s="117" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="D5" s="47">
         <v>1</v>
@@ -31146,7 +31385,7 @@
         <v>136</v>
       </c>
       <c r="X1" s="124" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -31154,10 +31393,10 @@
         <v>205</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="D2" s="30">
         <v>46226</v>
@@ -31179,13 +31418,13 @@
         <v>0</v>
       </c>
       <c r="M2" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N2" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="O2" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O2" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P2" s="12" t="s">
         <v>39</v>
@@ -31220,10 +31459,10 @@
         <v>206</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="D3" s="30">
         <v>46226</v>
@@ -31235,7 +31474,7 @@
         <v>25</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H3" s="30">
         <v>46242</v>
@@ -31249,13 +31488,13 @@
         <v>0</v>
       </c>
       <c r="M3" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N3" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N3" s="44" t="s">
+      <c r="O3" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O3" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P3" s="12" t="s">
         <v>39</v>
@@ -31290,10 +31529,10 @@
         <v>207</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D4" s="30">
         <v>46226</v>
@@ -31305,13 +31544,13 @@
         <v>390</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H4" s="30">
         <v>46248</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="J4" s="12"/>
       <c r="K4" s="13">
@@ -31321,13 +31560,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N4" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N4" s="44" t="s">
+      <c r="O4" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O4" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P4" s="12" t="s">
         <v>39</v>
@@ -31362,10 +31601,10 @@
         <v>208</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D5" s="30">
         <v>46226</v>
@@ -31377,7 +31616,7 @@
         <v>391</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H5" s="30">
         <v>46264</v>
@@ -31393,13 +31632,13 @@
         <v>0</v>
       </c>
       <c r="M5" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N5" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N5" s="44" t="s">
+      <c r="O5" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O5" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P5" s="12" t="s">
         <v>39</v>
@@ -31434,10 +31673,10 @@
         <v>209</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D6" s="30">
         <v>46226</v>
@@ -31449,7 +31688,7 @@
         <v>392</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H6" s="30">
         <v>46264</v>
@@ -31465,13 +31704,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N6" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N6" s="44" t="s">
+      <c r="O6" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O6" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P6" s="12" t="s">
         <v>39</v>
@@ -31506,10 +31745,10 @@
         <v>210</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D7" s="30">
         <v>46226</v>
@@ -31521,7 +31760,7 @@
         <v>395</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H7" s="30">
         <v>46417</v>
@@ -31537,13 +31776,13 @@
         <v>0</v>
       </c>
       <c r="M7" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N7" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N7" s="44" t="s">
+      <c r="O7" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O7" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P7" s="12" t="s">
         <v>39</v>
@@ -31578,10 +31817,10 @@
         <v>211</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D8" s="30">
         <v>46226</v>
@@ -31593,7 +31832,7 @@
         <v>393</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H8" s="30">
         <v>46537</v>
@@ -31609,13 +31848,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N8" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N8" s="44" t="s">
+      <c r="O8" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O8" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P8" s="12" t="s">
         <v>39</v>
@@ -31650,10 +31889,10 @@
         <v>212</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D9" s="30">
         <v>46226</v>
@@ -31665,7 +31904,7 @@
         <v>397</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H9" s="30">
         <v>46264</v>
@@ -31681,13 +31920,13 @@
         <v>0</v>
       </c>
       <c r="M9" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N9" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N9" s="44" t="s">
+      <c r="O9" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O9" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P9" s="12" t="s">
         <v>39</v>
@@ -33821,7 +34060,7 @@
     </row>
     <row r="51" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="48" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B51" s="56" t="s">
         <v>394</v>
@@ -33863,7 +34102,7 @@
     </row>
     <row r="52" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="48" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B52" s="56" t="s">
         <v>331</v>
@@ -33905,7 +34144,7 @@
     </row>
     <row r="53" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="48" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="B53" s="56" t="s">
         <v>396</v>
@@ -33947,7 +34186,7 @@
     </row>
     <row r="54" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="48" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="B54" s="56" t="s">
         <v>332</v>
@@ -33989,7 +34228,7 @@
     </row>
     <row r="55" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="48" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="B55" s="56" t="s">
         <v>333</v>
@@ -34033,7 +34272,7 @@
     </row>
     <row r="56" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="48" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B56" s="56" t="s">
         <v>334</v>
@@ -34075,7 +34314,7 @@
     </row>
     <row r="57" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="48" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="B57" s="56" t="s">
         <v>335</v>
@@ -34117,7 +34356,7 @@
     </row>
     <row r="58" spans="1:24" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="48" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B58" s="56" t="s">
         <v>336</v>
@@ -34916,7 +35155,7 @@
         <v>136</v>
       </c>
       <c r="Y1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -34927,7 +35166,7 @@
         <v>150</v>
       </c>
       <c r="C2" s="47" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="D2" s="30">
         <v>46226</v>
@@ -34949,13 +35188,13 @@
         <v>0</v>
       </c>
       <c r="M2" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N2" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="O2" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O2" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P2" s="47" t="s">
         <v>39</v>
@@ -34964,7 +35203,7 @@
         <v>28</v>
       </c>
       <c r="R2" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S2" s="47" t="s">
         <v>29</v>
@@ -34993,10 +35232,10 @@
         <v>238</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="C3" s="47" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="D3" s="30">
         <v>46211</v>
@@ -35008,7 +35247,7 @@
         <v>25</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H3" s="30">
         <v>46242</v>
@@ -35022,13 +35261,13 @@
         <v>0</v>
       </c>
       <c r="M3" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N3" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N3" s="44" t="s">
+      <c r="O3" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O3" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P3" s="47" t="s">
         <v>39</v>
@@ -35037,7 +35276,7 @@
         <v>28</v>
       </c>
       <c r="R3" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S3" s="47" t="s">
         <v>29</v>
@@ -35066,10 +35305,10 @@
         <v>239</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="D4" s="30">
         <v>46211</v>
@@ -35081,13 +35320,13 @@
         <v>390</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H4" s="30">
         <v>46248</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="J4" s="12"/>
       <c r="K4" s="13">
@@ -35097,13 +35336,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N4" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N4" s="44" t="s">
+      <c r="O4" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O4" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P4" s="47" t="s">
         <v>39</v>
@@ -35112,7 +35351,7 @@
         <v>28</v>
       </c>
       <c r="R4" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S4" s="47" t="s">
         <v>29</v>
@@ -35141,10 +35380,10 @@
         <v>240</v>
       </c>
       <c r="B5" s="53" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C5" s="47" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="D5" s="30">
         <v>46211</v>
@@ -35156,7 +35395,7 @@
         <v>391</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H5" s="30">
         <v>46264</v>
@@ -35172,13 +35411,13 @@
         <v>0</v>
       </c>
       <c r="M5" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N5" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N5" s="44" t="s">
+      <c r="O5" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O5" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P5" s="47" t="s">
         <v>39</v>
@@ -35187,7 +35426,7 @@
         <v>28</v>
       </c>
       <c r="R5" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S5" s="47" t="s">
         <v>29</v>
@@ -35216,10 +35455,10 @@
         <v>241</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="C6" s="47" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D6" s="30">
         <v>46211</v>
@@ -35231,7 +35470,7 @@
         <v>392</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H6" s="30">
         <v>46264</v>
@@ -35247,13 +35486,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N6" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N6" s="44" t="s">
+      <c r="O6" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O6" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P6" s="47" t="s">
         <v>39</v>
@@ -35262,7 +35501,7 @@
         <v>28</v>
       </c>
       <c r="R6" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S6" s="47" t="s">
         <v>29</v>
@@ -35291,10 +35530,10 @@
         <v>242</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C7" s="47" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="D7" s="30">
         <v>46211</v>
@@ -35306,7 +35545,7 @@
         <v>395</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H7" s="30">
         <v>46417</v>
@@ -35322,13 +35561,13 @@
         <v>0</v>
       </c>
       <c r="M7" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N7" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N7" s="44" t="s">
+      <c r="O7" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O7" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P7" s="47" t="s">
         <v>39</v>
@@ -35337,7 +35576,7 @@
         <v>28</v>
       </c>
       <c r="R7" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S7" s="47" t="s">
         <v>29</v>
@@ -35366,10 +35605,10 @@
         <v>243</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="C8" s="47" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D8" s="30">
         <v>46211</v>
@@ -35381,7 +35620,7 @@
         <v>393</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H8" s="30">
         <v>46537</v>
@@ -35397,13 +35636,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N8" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N8" s="44" t="s">
+      <c r="O8" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O8" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P8" s="47" t="s">
         <v>39</v>
@@ -35412,7 +35651,7 @@
         <v>28</v>
       </c>
       <c r="R8" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S8" s="47" t="s">
         <v>29</v>
@@ -35441,10 +35680,10 @@
         <v>244</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C9" s="47" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="D9" s="30">
         <v>46211</v>
@@ -35456,7 +35695,7 @@
         <v>397</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="H9" s="30">
         <v>46233</v>
@@ -35472,13 +35711,13 @@
         <v>0</v>
       </c>
       <c r="M9" s="44" t="s">
+        <v>840</v>
+      </c>
+      <c r="N9" s="44" t="s">
         <v>841</v>
       </c>
-      <c r="N9" s="44" t="s">
+      <c r="O9" s="44" t="s">
         <v>842</v>
-      </c>
-      <c r="O9" s="44" t="s">
-        <v>843</v>
       </c>
       <c r="P9" s="47" t="s">
         <v>39</v>
@@ -35487,7 +35726,7 @@
         <v>28</v>
       </c>
       <c r="R9" s="47" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="S9" s="47" t="s">
         <v>29</v>
@@ -37763,7 +38002,7 @@
     </row>
     <row r="52" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="47" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B52" s="47" t="s">
         <v>330</v>
@@ -37808,7 +38047,7 @@
     </row>
     <row r="53" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="47" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="B53" s="78" t="s">
         <v>331</v>
@@ -37853,7 +38092,7 @@
     </row>
     <row r="54" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="47" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B54" s="47" t="s">
         <v>332</v>
@@ -37900,7 +38139,7 @@
     </row>
     <row r="55" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="47" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B55" s="78" t="s">
         <v>333</v>
@@ -37945,7 +38184,7 @@
     </row>
     <row r="56" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="47" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="B56" s="47" t="s">
         <v>334</v>
@@ -37990,7 +38229,7 @@
     </row>
     <row r="57" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="47" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B57" s="78" t="s">
         <v>335</v>
@@ -38035,7 +38274,7 @@
     </row>
     <row r="58" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="47" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B58" s="47" t="s">
         <v>336</v>
@@ -39102,18 +39341,18 @@
         <v>136</v>
       </c>
       <c r="E1" s="119" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="47" t="s">
+        <v>785</v>
+      </c>
+      <c r="B2" s="47" t="s">
         <v>786</v>
       </c>
-      <c r="B2" s="47" t="s">
-        <v>787</v>
-      </c>
       <c r="C2" s="62" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="D2" s="47" t="s">
         <v>272</v>
@@ -39124,13 +39363,13 @@
     </row>
     <row r="3" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B3" s="47" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="C3" s="62" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D3" s="47" t="s">
         <v>272</v>
@@ -39141,13 +39380,13 @@
     </row>
     <row r="4" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="47" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="C4" s="62" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="D4" s="47" t="s">
         <v>272</v>
@@ -39158,13 +39397,13 @@
     </row>
     <row r="5" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="B5" s="47" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="C5" s="62" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D5" s="47" t="s">
         <v>272</v>
@@ -39175,13 +39414,13 @@
     </row>
     <row r="6" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="47" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B6" s="47" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="C6" s="62" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="D6" s="47" t="s">
         <v>272</v>
@@ -39192,13 +39431,13 @@
     </row>
     <row r="7" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="47" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B7" s="47" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="C7" s="62" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>272</v>
@@ -39209,13 +39448,13 @@
     </row>
     <row r="8" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="47" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B8" s="47" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>272</v>
@@ -39226,13 +39465,13 @@
     </row>
     <row r="9" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="47" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B9" s="47" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="D9" s="47" t="s">
         <v>272</v>
@@ -39243,13 +39482,13 @@
     </row>
     <row r="10" spans="1:5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="47" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="B10" s="47" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="C10" s="62" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="D10" s="47" t="s">
         <v>272</v>

</xml_diff>